<commit_message>
chore(mom): update minutes of meeting for 2026-09-14
Updated the Excel file containing the minutes of the meeting held on September 14, 2026. This includes any new notes or changes discussed during the meeting.
</commit_message>
<xml_diff>
--- a/docs/minutes-of-meeting/mom-20260914.xlsx
+++ b/docs/minutes-of-meeting/mom-20260914.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\medcal\docs\minutes-of-meeting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B6BD6E3-9995-4109-B811-4071366FDA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97C6D4F-ED90-4683-BF5C-5E2DDF755E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0F5C309D-145E-4108-8C74-C8953C6BB10A}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Minutes Of Meeting (Demo) 14/09/2026</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>sebaiknya buat 1 fungsi yg bisa mengatur level keketatan system, misalnya: Moderate / Strict dan ini berlaku ke semua fungsi mulai</t>
+  </si>
+  <si>
+    <t>Ada beberapa parameter yang mesti diisi dengan range (awal-akhir) sehingga tidak perlu perulangan saat kalibrasi (pengukuran)</t>
   </si>
 </sst>
 </file>
@@ -494,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{101CD0AC-F4DB-4567-BEC3-AF301E7F007D}">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.109375" bestFit="1" customWidth="1"/>
@@ -676,6 +679,15 @@
       </c>
       <c r="C24" s="2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="3" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>10</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add space for descriptions in mom-20260914.xlsx
</commit_message>
<xml_diff>
--- a/docs/minutes-of-meeting/mom-20260914.xlsx
+++ b/docs/minutes-of-meeting/mom-20260914.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\medcal\docs\minutes-of-meeting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A97C6D4F-ED90-4683-BF5C-5E2DDF755E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C908C2F1-33F9-4727-9165-7E8D0AD55596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0F5C309D-145E-4108-8C74-C8953C6BB10A}"/>
   </bookViews>
@@ -502,7 +502,7 @@
   <cols>
     <col min="1" max="1" width="3.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="118.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="131.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="144.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.35">

</xml_diff>